<commit_message>
v0.2 shell script finalized, naming conventions, Interessenwoche Excel update
</commit_message>
<xml_diff>
--- a/Interessenwochen/Wn_Gf_Sommer_2024/Weitere Dokumente/Interessenwoche_Listen_FS2024.xlsx
+++ b/Interessenwochen/Wn_Gf_Sommer_2024/Weitere Dokumente/Interessenwoche_Listen_FS2024.xlsx
@@ -1,19 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10609"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10609"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cyrilwendl/LeeTeX/Interessenwochen/Wn_Gf_Sommer_2024/Weitere Dokumente/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97C30531-4A44-1D42-971F-AFB77232C6FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DC13B7D-91D1-894F-9A7C-8DB243A57022}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Table 1" sheetId="1" r:id="rId1"/>
+    <sheet name="TN" sheetId="1" r:id="rId1"/>
+    <sheet name="Bewertung Projekte" sheetId="2" r:id="rId2"/>
+    <sheet name="Kosten" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="109">
   <si>
     <r>
       <rPr>
@@ -851,6 +853,69 @@
   </si>
   <si>
     <t>GA</t>
+  </si>
+  <si>
+    <t>Bewertungskriterium</t>
+  </si>
+  <si>
+    <t>Punkte / Kriterium</t>
+  </si>
+  <si>
+    <t>Tabellen</t>
+  </si>
+  <si>
+    <t>Listen (ol UND ul)</t>
+  </si>
+  <si>
+    <t>Zitate</t>
+  </si>
+  <si>
+    <t>Links</t>
+  </si>
+  <si>
+    <t>3 weitere HTML-Tags</t>
+  </si>
+  <si>
+    <t>Stylesheet</t>
+  </si>
+  <si>
+    <t>Gesamt-Punkte</t>
+  </si>
+  <si>
+    <t>Mention</t>
+  </si>
+  <si>
+    <t>Gruppe</t>
+  </si>
+  <si>
+    <t>Latex Template</t>
+  </si>
+  <si>
+    <t>Platz</t>
+  </si>
+  <si>
+    <t>Inhalt gut verstanden &amp; präsentiert</t>
+  </si>
+  <si>
+    <t>Bonus: Favicon</t>
+  </si>
+  <si>
+    <t>Bonus: Design</t>
+  </si>
+  <si>
+    <t>Bonus: JavaScript / Interaktiv</t>
+  </si>
+  <si>
+    <t>Bonus: Vektor-Grafiken</t>
+  </si>
+  <si>
+    <t>CHF 27.70 bezahlt</t>
+  </si>
+  <si>
+    <t>Durchführung 1</t>
+  </si>
+  <si>
+    <t>Durchführung 2</t>
   </si>
 </sst>
 </file>
@@ -909,12 +974,24 @@
       <family val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="3">
@@ -950,48 +1027,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="3"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" indent="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="3"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" indent="2" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -1003,6 +1041,75 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="3"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" indent="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="3"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" indent="2" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="3"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" indent="3"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="3"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" indent="3"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
@@ -1310,633 +1417,1989 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:AD35"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="8" customWidth="1"/>
-    <col min="2" max="2" width="26.59765625" customWidth="1"/>
-    <col min="3" max="3" width="25.59765625" customWidth="1"/>
-    <col min="4" max="4" width="32.59765625" customWidth="1"/>
-    <col min="5" max="5" width="21.796875" customWidth="1"/>
-    <col min="6" max="6" width="11.59765625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.19921875" customWidth="1"/>
-    <col min="8" max="8" width="11.796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8" style="7" customWidth="1"/>
+    <col min="2" max="4" width="19.59765625" style="7" customWidth="1"/>
+    <col min="5" max="5" width="48.3984375" style="26" customWidth="1"/>
+    <col min="6" max="6" width="11.19921875" style="26" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22.3984375" style="26" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.19921875" style="26" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.19921875" style="7" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="21.796875" style="7" customWidth="1"/>
+    <col min="11" max="11" width="11.59765625" style="7" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="30" style="7" customWidth="1"/>
+    <col min="13" max="21" width="25.19921875" style="7" customWidth="1"/>
+    <col min="22" max="25" width="9" style="7"/>
+    <col min="26" max="26" width="9.59765625" style="7" bestFit="1" customWidth="1"/>
+    <col min="27" max="29" width="9" style="7"/>
+    <col min="30" max="30" width="10.19921875" style="7" customWidth="1"/>
+    <col min="31" max="31" width="11.796875" style="7" bestFit="1" customWidth="1"/>
+    <col min="32" max="16384" width="9" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="34" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="13" t="s">
+    <row r="1" spans="1:30" ht="34" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-    </row>
-    <row r="2" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="3" t="s">
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
+      <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
+      <c r="L1" s="8"/>
+    </row>
+    <row r="2" spans="1:30" ht="17" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A2" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="E2" s="22" t="s">
+        <v>99</v>
+      </c>
+      <c r="F2" s="23" t="s">
+        <v>100</v>
+      </c>
+      <c r="G2" s="22" t="s">
+        <v>100</v>
+      </c>
+      <c r="H2" s="22" t="s">
+        <v>97</v>
+      </c>
+      <c r="I2" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="J2" s="13" t="s">
         <v>77</v>
       </c>
-      <c r="F2" s="17" t="s">
+      <c r="K2" s="14" t="s">
         <v>86</v>
       </c>
-      <c r="G2" s="17"/>
-      <c r="H2" s="17" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="6">
-        <v>1</v>
-      </c>
-      <c r="B3" s="7" t="s">
+      <c r="L2" s="14"/>
+      <c r="M2" s="8"/>
+      <c r="N2" s="8"/>
+      <c r="O2" s="8"/>
+      <c r="P2" s="8"/>
+      <c r="Q2" s="8"/>
+      <c r="R2" s="8"/>
+      <c r="S2" s="8"/>
+      <c r="T2" s="8"/>
+      <c r="U2" s="8"/>
+      <c r="V2" s="8"/>
+      <c r="W2" s="8"/>
+      <c r="X2" s="8"/>
+      <c r="Y2" s="8"/>
+      <c r="Z2" s="8"/>
+      <c r="AA2" s="8"/>
+      <c r="AB2" s="8"/>
+      <c r="AC2" s="8"/>
+      <c r="AD2" s="14"/>
+    </row>
+    <row r="3" spans="1:30" ht="17" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A3" s="15">
+        <v>1</v>
+      </c>
+      <c r="B3" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="D3" s="17">
+        <v>4</v>
+      </c>
+      <c r="E3" s="24" t="str">
+        <f>C3&amp;" "&amp;B3 &amp;"/"&amp;G3&amp;"/"&amp;H3&amp;","</f>
+        <v>Loris Alexander Amacker/2. Platz/{herausragendes },</v>
+      </c>
+      <c r="F3" s="25">
+        <f>_xlfn.XLOOKUP(D3,'Bewertung Projekte'!$C$3:$H$3,'Bewertung Projekte'!$C$16:$H$16)</f>
+        <v>2</v>
+      </c>
+      <c r="G3" s="24" t="str">
+        <f>IF(F3&lt;4,F3&amp;". Platz", "Honorable Mention")</f>
+        <v>2. Platz</v>
+      </c>
+      <c r="H3" s="24" t="str">
+        <f t="shared" ref="H3:H15" si="0">IF(ISERR(FIND("Platz",G3)),"","{herausragendes }")</f>
+        <v>{herausragendes }</v>
+      </c>
+      <c r="I3" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="11" t="s">
+      <c r="J3" s="19" t="s">
         <v>76</v>
       </c>
-      <c r="H3" s="15">
+    </row>
+    <row r="4" spans="1:30" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A4" s="15">
+        <v>2</v>
+      </c>
+      <c r="B4" s="16" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="17">
+        <v>2</v>
+      </c>
+      <c r="E4" s="24" t="str">
+        <f>C4&amp;" "&amp;B4 &amp;"/"&amp;G4&amp;"/"&amp;H4&amp;","</f>
+        <v>Jan Sebastian Baik/Honorable Mention/,</v>
+      </c>
+      <c r="F4" s="25">
+        <f>_xlfn.XLOOKUP(D4,'Bewertung Projekte'!$C$3:$H$3,'Bewertung Projekte'!$C$16:$H$16)</f>
         <v>5</v>
       </c>
-      <c r="I3" s="14" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="6">
+      <c r="G4" s="24" t="str">
+        <f t="shared" ref="G4:G16" si="1">IF(F4&lt;4,F4&amp;". Platz", "Honorable Mention")</f>
+        <v>Honorable Mention</v>
+      </c>
+      <c r="H4" s="24" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="I4" s="18" t="s">
+        <v>10</v>
+      </c>
+      <c r="J4" s="19" t="s">
+        <v>76</v>
+      </c>
+      <c r="K4" s="8" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="5" spans="1:30" ht="17" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A5" s="15">
+        <v>3</v>
+      </c>
+      <c r="B5" s="16" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="17">
+        <v>1</v>
+      </c>
+      <c r="E5" s="24" t="str">
+        <f>C5&amp;" "&amp;B5 &amp;"/"&amp;G5&amp;"/"&amp;H5&amp;","</f>
+        <v>Dennis Beck/3. Platz/{herausragendes },</v>
+      </c>
+      <c r="F5" s="25">
+        <f>_xlfn.XLOOKUP(D5,'Bewertung Projekte'!$C$3:$H$3,'Bewertung Projekte'!$C$16:$H$16)</f>
+        <v>3</v>
+      </c>
+      <c r="G5" s="24" t="str">
+        <f t="shared" si="1"/>
+        <v>3. Platz</v>
+      </c>
+      <c r="H5" s="24" t="str">
+        <f t="shared" si="0"/>
+        <v>{herausragendes }</v>
+      </c>
+      <c r="I5" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="J5" s="19" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="6" spans="1:30" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A6" s="15">
+        <v>4</v>
+      </c>
+      <c r="B6" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="17" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" s="17">
+        <v>5</v>
+      </c>
+      <c r="E6" s="24" t="str">
+        <f>C6&amp;" "&amp;B6 &amp;"/"&amp;G6&amp;"/"&amp;H6&amp;","</f>
+        <v>Florian Boss/1. Platz/{herausragendes },</v>
+      </c>
+      <c r="F6" s="25">
+        <f>_xlfn.XLOOKUP(D6,'Bewertung Projekte'!$C$3:$H$3,'Bewertung Projekte'!$C$16:$H$16)</f>
+        <v>1</v>
+      </c>
+      <c r="G6" s="24" t="str">
+        <f t="shared" si="1"/>
+        <v>1. Platz</v>
+      </c>
+      <c r="H6" s="24" t="str">
+        <f t="shared" si="0"/>
+        <v>{herausragendes }</v>
+      </c>
+      <c r="I6" s="18" t="s">
+        <v>15</v>
+      </c>
+      <c r="J6" s="19" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="7" spans="1:30" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A7" s="15">
+        <v>5</v>
+      </c>
+      <c r="B7" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" s="17" t="s">
+        <v>17</v>
+      </c>
+      <c r="D7" s="17">
+        <v>5</v>
+      </c>
+      <c r="E7" s="24" t="str">
+        <f>C7&amp;" "&amp;B7 &amp;"/"&amp;G7&amp;"/"&amp;H7&amp;","</f>
+        <v>Matteo Esteban Ceccon/1. Platz/{herausragendes },</v>
+      </c>
+      <c r="F7" s="25">
+        <f>_xlfn.XLOOKUP(D7,'Bewertung Projekte'!$C$3:$H$3,'Bewertung Projekte'!$C$16:$H$16)</f>
+        <v>1</v>
+      </c>
+      <c r="G7" s="24" t="str">
+        <f t="shared" si="1"/>
+        <v>1. Platz</v>
+      </c>
+      <c r="H7" s="24" t="str">
+        <f t="shared" si="0"/>
+        <v>{herausragendes }</v>
+      </c>
+      <c r="I7" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="J7" s="19" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="8" spans="1:30" ht="17" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A8" s="15">
+        <v>6</v>
+      </c>
+      <c r="B8" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="17">
+        <v>4</v>
+      </c>
+      <c r="E8" s="24" t="str">
+        <f>C8&amp;" "&amp;B8 &amp;"/"&amp;G8&amp;"/"&amp;H8&amp;","</f>
+        <v>Marcel Debrunner/2. Platz/{herausragendes },</v>
+      </c>
+      <c r="F8" s="25">
+        <f>_xlfn.XLOOKUP(D8,'Bewertung Projekte'!$C$3:$H$3,'Bewertung Projekte'!$C$16:$H$16)</f>
         <v>2</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="G8" s="24" t="str">
+        <f t="shared" si="1"/>
+        <v>2. Platz</v>
+      </c>
+      <c r="H8" s="24" t="str">
+        <f t="shared" si="0"/>
+        <v>{herausragendes }</v>
+      </c>
+      <c r="I8" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="J8" s="19" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="9" spans="1:30" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A9" s="15">
+        <v>7</v>
+      </c>
+      <c r="B9" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="D9" s="17">
+        <v>3</v>
+      </c>
+      <c r="E9" s="24" t="str">
+        <f>C9&amp;" "&amp;B9 &amp;"/"&amp;G9&amp;"/"&amp;H9&amp;","</f>
+        <v>Felix Fischer/Honorable Mention/,</v>
+      </c>
+      <c r="F9" s="25">
+        <f>_xlfn.XLOOKUP(D9,'Bewertung Projekte'!$C$3:$H$3,'Bewertung Projekte'!$C$16:$H$16)</f>
+        <v>6</v>
+      </c>
+      <c r="G9" s="24" t="str">
+        <f t="shared" si="1"/>
+        <v>Honorable Mention</v>
+      </c>
+      <c r="H9" s="24" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="I9" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="J9" s="19" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="10" spans="1:30" ht="17" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A10" s="15">
         <v>8</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="B10" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="D10" s="17">
+        <v>6</v>
+      </c>
+      <c r="E10" s="24" t="str">
+        <f>C10&amp;" "&amp;B10 &amp;"/"&amp;G10&amp;"/"&amp;H10&amp;","</f>
+        <v>Lina Flückiger/Honorable Mention/,</v>
+      </c>
+      <c r="F10" s="25">
+        <f>_xlfn.XLOOKUP(D10,'Bewertung Projekte'!$C$3:$H$3,'Bewertung Projekte'!$C$16:$H$16)</f>
+        <v>4</v>
+      </c>
+      <c r="G10" s="24" t="str">
+        <f t="shared" si="1"/>
+        <v>Honorable Mention</v>
+      </c>
+      <c r="H10" s="24" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="I10" s="18" t="s">
+        <v>15</v>
+      </c>
+      <c r="J10" s="19" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="11" spans="1:30" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A11" s="15">
         <v>9</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="B11" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="D11" s="17">
+        <v>6</v>
+      </c>
+      <c r="E11" s="24" t="str">
+        <f>C11&amp;" "&amp;B11 &amp;"/"&amp;G11&amp;"/"&amp;H11&amp;","</f>
+        <v>Beatrice Fullagar/Honorable Mention/,</v>
+      </c>
+      <c r="F11" s="25">
+        <f>_xlfn.XLOOKUP(D11,'Bewertung Projekte'!$C$3:$H$3,'Bewertung Projekte'!$C$16:$H$16)</f>
+        <v>4</v>
+      </c>
+      <c r="G11" s="24" t="str">
+        <f t="shared" si="1"/>
+        <v>Honorable Mention</v>
+      </c>
+      <c r="H11" s="24" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="I11" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="J11" s="19" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="12" spans="1:30" ht="17" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A12" s="21">
         <v>10</v>
       </c>
-      <c r="E4" s="11" t="s">
+      <c r="B12" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="D12" s="17">
+        <v>3</v>
+      </c>
+      <c r="E12" s="24" t="str">
+        <f>C12&amp;" "&amp;B12 &amp;"/"&amp;G12&amp;"/"&amp;H12&amp;","</f>
+        <v>Niclas Graf/Honorable Mention/,</v>
+      </c>
+      <c r="F12" s="25">
+        <f>_xlfn.XLOOKUP(D12,'Bewertung Projekte'!$C$3:$H$3,'Bewertung Projekte'!$C$16:$H$16)</f>
+        <v>6</v>
+      </c>
+      <c r="G12" s="24" t="str">
+        <f t="shared" si="1"/>
+        <v>Honorable Mention</v>
+      </c>
+      <c r="H12" s="24" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="I12" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="J12" s="19" t="s">
         <v>76</v>
       </c>
-      <c r="F4" s="14" t="s">
+    </row>
+    <row r="13" spans="1:30" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A13" s="21">
+        <v>11</v>
+      </c>
+      <c r="B13" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="D13" s="17">
+        <v>2</v>
+      </c>
+      <c r="E13" s="24" t="str">
+        <f>C13&amp;" "&amp;B13 &amp;"/"&amp;G13&amp;"/"&amp;H13&amp;","</f>
+        <v>Ikarus Knoblauch/Honorable Mention/,</v>
+      </c>
+      <c r="F13" s="25">
+        <f>_xlfn.XLOOKUP(D13,'Bewertung Projekte'!$C$3:$H$3,'Bewertung Projekte'!$C$16:$H$16)</f>
+        <v>5</v>
+      </c>
+      <c r="G13" s="24" t="str">
+        <f t="shared" si="1"/>
+        <v>Honorable Mention</v>
+      </c>
+      <c r="H13" s="24" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="I13" s="18" t="s">
+        <v>10</v>
+      </c>
+      <c r="J13" s="19" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="14" spans="1:30" ht="17" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A14" s="21">
+        <v>12</v>
+      </c>
+      <c r="B14" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="C14" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="D14" s="17">
+        <v>4</v>
+      </c>
+      <c r="E14" s="24" t="str">
+        <f>C14&amp;" "&amp;B14 &amp;"/"&amp;G14&amp;"/"&amp;H14&amp;","</f>
+        <v>Bernard Rognon/2. Platz/{herausragendes },</v>
+      </c>
+      <c r="F14" s="25">
+        <f>_xlfn.XLOOKUP(D14,'Bewertung Projekte'!$C$3:$H$3,'Bewertung Projekte'!$C$16:$H$16)</f>
+        <v>2</v>
+      </c>
+      <c r="G14" s="24" t="str">
+        <f t="shared" si="1"/>
+        <v>2. Platz</v>
+      </c>
+      <c r="H14" s="24" t="str">
+        <f t="shared" si="0"/>
+        <v>{herausragendes }</v>
+      </c>
+      <c r="I14" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="J14" s="19" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="15" spans="1:30" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A15" s="21">
+        <v>13</v>
+      </c>
+      <c r="B15" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="C15" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="D15" s="17">
+        <v>5</v>
+      </c>
+      <c r="E15" s="24" t="str">
+        <f>C15&amp;" "&amp;B15 &amp;"/"&amp;G15&amp;"/"&amp;H15&amp;","</f>
+        <v>Lenny Matteo Schmid/1. Platz/{herausragendes },</v>
+      </c>
+      <c r="F15" s="25">
+        <f>_xlfn.XLOOKUP(D15,'Bewertung Projekte'!$C$3:$H$3,'Bewertung Projekte'!$C$16:$H$16)</f>
+        <v>1</v>
+      </c>
+      <c r="G15" s="24" t="str">
+        <f t="shared" si="1"/>
+        <v>1. Platz</v>
+      </c>
+      <c r="H15" s="24" t="str">
+        <f t="shared" si="0"/>
+        <v>{herausragendes }</v>
+      </c>
+      <c r="I15" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="J15" s="19" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="16" spans="1:30" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A16" s="21">
+        <v>14</v>
+      </c>
+      <c r="B16" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="C16" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="D16" s="17">
+        <v>1</v>
+      </c>
+      <c r="E16" s="24" t="str">
+        <f>C16&amp;" "&amp;B16 &amp;"/"&amp;G16&amp;"/"&amp;H16&amp;","</f>
+        <v>Julius Schöner/3. Platz/{herausragendes },</v>
+      </c>
+      <c r="F16" s="25">
+        <f>_xlfn.XLOOKUP(D16,'Bewertung Projekte'!$C$3:$H$3,'Bewertung Projekte'!$C$16:$H$16)</f>
+        <v>3</v>
+      </c>
+      <c r="G16" s="24" t="str">
+        <f t="shared" si="1"/>
+        <v>3. Platz</v>
+      </c>
+      <c r="H16" s="24" t="str">
+        <f>IF(ISERR(FIND("Platz",G16)),"","{herausragendes }")</f>
+        <v>{herausragendes }</v>
+      </c>
+      <c r="I16" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="J16" s="19" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="48" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A17" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B17" s="6"/>
+      <c r="C17" s="6"/>
+      <c r="D17" s="6"/>
+      <c r="E17" s="6"/>
+      <c r="F17" s="6"/>
+      <c r="G17" s="6"/>
+      <c r="H17" s="6"/>
+      <c r="I17" s="6"/>
+      <c r="J17" s="6"/>
+    </row>
+    <row r="18" spans="1:11" ht="17" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A18" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="C18" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="D18" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="E18" s="22" t="s">
+        <v>99</v>
+      </c>
+      <c r="F18" s="23" t="s">
+        <v>100</v>
+      </c>
+      <c r="G18" s="22" t="s">
+        <v>100</v>
+      </c>
+      <c r="H18" s="22" t="s">
+        <v>97</v>
+      </c>
+      <c r="I18" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="J18" s="13" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="17" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A19" s="15">
+        <v>1</v>
+      </c>
+      <c r="B19" s="16" t="s">
+        <v>38</v>
+      </c>
+      <c r="C19" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="D19" s="17">
+        <v>1</v>
+      </c>
+      <c r="E19" s="24" t="str">
+        <f>C19&amp;" "&amp;B19 &amp;"/1. Platz,"</f>
+        <v>Livio Adorni/1. Platz,</v>
+      </c>
+      <c r="F19" s="25">
+        <f>_xlfn.XLOOKUP(D19,'Bewertung Projekte'!$C$23:$J$23,'Bewertung Projekte'!$C$36:$J$36)</f>
+        <v>1</v>
+      </c>
+      <c r="G19" s="24" t="str">
+        <f>IF(F19&lt;4,F19&amp;". Platz", "Honorable Mention")</f>
+        <v>1. Platz</v>
+      </c>
+      <c r="H19" s="24" t="str">
+        <f t="shared" ref="H19:H35" si="2">IF(ISERR(FIND("Platz",G19)),"","{herausragendes }")</f>
+        <v>{herausragendes }</v>
+      </c>
+      <c r="I19" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="J19" s="20"/>
+    </row>
+    <row r="20" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A20" s="15">
+        <v>2</v>
+      </c>
+      <c r="B20" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C20" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="D20" s="17">
+        <v>5</v>
+      </c>
+      <c r="E20" s="24" t="str">
+        <f t="shared" ref="E20:E35" si="3">C20&amp;" "&amp;B20 &amp;"/1. Platz,"</f>
+        <v>Jonas Billeter/1. Platz,</v>
+      </c>
+      <c r="F20" s="25">
+        <f>_xlfn.XLOOKUP(D20,'Bewertung Projekte'!$C$23:$J$23,'Bewertung Projekte'!$C$36:$J$36)</f>
+        <v>3</v>
+      </c>
+      <c r="G20" s="24" t="str">
+        <f t="shared" ref="G20:G35" si="4">IF(F20&lt;4,F20&amp;". Platz", "Honorable Mention")</f>
+        <v>3. Platz</v>
+      </c>
+      <c r="H20" s="24" t="str">
+        <f t="shared" si="2"/>
+        <v>{herausragendes }</v>
+      </c>
+      <c r="I20" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="J20" s="20"/>
+    </row>
+    <row r="21" spans="1:11" ht="17" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A21" s="15">
+        <v>3</v>
+      </c>
+      <c r="B21" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="C21" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="D21" s="17">
+        <v>3</v>
+      </c>
+      <c r="E21" s="24" t="str">
+        <f t="shared" si="3"/>
+        <v>Timo Bloch/1. Platz,</v>
+      </c>
+      <c r="F21" s="25">
+        <f>_xlfn.XLOOKUP(D21,'Bewertung Projekte'!$C$23:$J$23,'Bewertung Projekte'!$C$36:$J$36)</f>
+        <v>5</v>
+      </c>
+      <c r="G21" s="24" t="str">
+        <f t="shared" si="4"/>
+        <v>Honorable Mention</v>
+      </c>
+      <c r="H21" s="24" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="I21" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="J21" s="20"/>
+    </row>
+    <row r="22" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A22" s="15">
+        <v>4</v>
+      </c>
+      <c r="B22" s="16" t="s">
+        <v>47</v>
+      </c>
+      <c r="C22" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="D22" s="17">
+        <v>3</v>
+      </c>
+      <c r="E22" s="24" t="str">
+        <f t="shared" si="3"/>
+        <v>Joris Boogman/1. Platz,</v>
+      </c>
+      <c r="F22" s="25">
+        <f>_xlfn.XLOOKUP(D22,'Bewertung Projekte'!$C$23:$J$23,'Bewertung Projekte'!$C$36:$J$36)</f>
+        <v>5</v>
+      </c>
+      <c r="G22" s="24" t="str">
+        <f t="shared" si="4"/>
+        <v>Honorable Mention</v>
+      </c>
+      <c r="H22" s="24" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="I22" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="J22" s="20"/>
+    </row>
+    <row r="23" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A23" s="15">
+        <v>5</v>
+      </c>
+      <c r="B23" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="C23" s="17" t="s">
+        <v>51</v>
+      </c>
+      <c r="D23" s="17">
+        <v>1</v>
+      </c>
+      <c r="E23" s="24" t="str">
+        <f t="shared" si="3"/>
+        <v>Tim Bretscher/1. Platz,</v>
+      </c>
+      <c r="F23" s="25">
+        <f>_xlfn.XLOOKUP(D23,'Bewertung Projekte'!$C$23:$J$23,'Bewertung Projekte'!$C$36:$J$36)</f>
+        <v>1</v>
+      </c>
+      <c r="G23" s="24" t="str">
+        <f t="shared" si="4"/>
+        <v>1. Platz</v>
+      </c>
+      <c r="H23" s="24" t="str">
+        <f t="shared" si="2"/>
+        <v>{herausragendes }</v>
+      </c>
+      <c r="I23" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="J23" s="20"/>
+    </row>
+    <row r="24" spans="1:11" ht="17" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A24" s="15">
+        <v>6</v>
+      </c>
+      <c r="B24" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="C24" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="D24" s="17">
+        <v>2</v>
+      </c>
+      <c r="E24" s="24" t="str">
+        <f t="shared" si="3"/>
+        <v>Sophie Joy Haltinner/1. Platz,</v>
+      </c>
+      <c r="F24" s="25">
+        <f>_xlfn.XLOOKUP(D24,'Bewertung Projekte'!$C$23:$J$23,'Bewertung Projekte'!$C$36:$J$36)</f>
+        <v>4</v>
+      </c>
+      <c r="G24" s="24" t="str">
+        <f t="shared" si="4"/>
+        <v>Honorable Mention</v>
+      </c>
+      <c r="H24" s="24" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="I24" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="J24" s="20"/>
+    </row>
+    <row r="25" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A25" s="15">
+        <v>7</v>
+      </c>
+      <c r="B25" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="C25" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="D25" s="17">
+        <v>8</v>
+      </c>
+      <c r="E25" s="24" t="str">
+        <f t="shared" si="3"/>
+        <v>Julien Hirsiger/1. Platz,</v>
+      </c>
+      <c r="F25" s="25">
+        <f>_xlfn.XLOOKUP(D25,'Bewertung Projekte'!$C$23:$J$23,'Bewertung Projekte'!$C$36:$J$36)</f>
+        <v>7</v>
+      </c>
+      <c r="G25" s="24" t="str">
+        <f t="shared" si="4"/>
+        <v>Honorable Mention</v>
+      </c>
+      <c r="H25" s="24" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="I25" s="18" t="s">
+        <v>56</v>
+      </c>
+      <c r="J25" s="20"/>
+    </row>
+    <row r="26" spans="1:11" ht="17" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A26" s="15">
+        <v>8</v>
+      </c>
+      <c r="B26" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="C26" s="17" t="s">
+        <v>58</v>
+      </c>
+      <c r="D26" s="17">
+        <v>1</v>
+      </c>
+      <c r="E26" s="24" t="str">
+        <f t="shared" si="3"/>
+        <v>Clemens Holzschuster/1. Platz,</v>
+      </c>
+      <c r="F26" s="25">
+        <f>_xlfn.XLOOKUP(D26,'Bewertung Projekte'!$C$23:$J$23,'Bewertung Projekte'!$C$36:$J$36)</f>
+        <v>1</v>
+      </c>
+      <c r="G26" s="24" t="str">
+        <f t="shared" si="4"/>
+        <v>1. Platz</v>
+      </c>
+      <c r="H26" s="24" t="str">
+        <f t="shared" si="2"/>
+        <v>{herausragendes }</v>
+      </c>
+      <c r="I26" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="J26" s="20"/>
+    </row>
+    <row r="27" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A27" s="15">
+        <v>9</v>
+      </c>
+      <c r="B27" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="C27" s="17" t="s">
+        <v>60</v>
+      </c>
+      <c r="D27" s="17">
+        <v>6</v>
+      </c>
+      <c r="E27" s="24" t="str">
+        <f t="shared" si="3"/>
+        <v>Carpie Kasongo Basuiye/1. Platz,</v>
+      </c>
+      <c r="F27" s="25">
+        <f>_xlfn.XLOOKUP(D27,'Bewertung Projekte'!$C$23:$J$23,'Bewertung Projekte'!$C$36:$J$36)</f>
+        <v>8</v>
+      </c>
+      <c r="G27" s="24" t="str">
+        <f t="shared" si="4"/>
+        <v>Honorable Mention</v>
+      </c>
+      <c r="H27" s="24" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="I27" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="J27" s="20"/>
+    </row>
+    <row r="28" spans="1:11" ht="17" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A28" s="21">
+        <v>10</v>
+      </c>
+      <c r="B28" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="C28" s="17" t="s">
+        <v>62</v>
+      </c>
+      <c r="D28" s="17">
+        <v>6</v>
+      </c>
+      <c r="E28" s="24" t="str">
+        <f t="shared" si="3"/>
+        <v>Iman Lee/1. Platz,</v>
+      </c>
+      <c r="F28" s="25">
+        <f>_xlfn.XLOOKUP(D28,'Bewertung Projekte'!$C$23:$J$23,'Bewertung Projekte'!$C$36:$J$36)</f>
+        <v>8</v>
+      </c>
+      <c r="G28" s="24" t="str">
+        <f t="shared" si="4"/>
+        <v>Honorable Mention</v>
+      </c>
+      <c r="H28" s="24" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="I28" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="J28" s="20"/>
+    </row>
+    <row r="29" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A29" s="21">
+        <v>11</v>
+      </c>
+      <c r="B29" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="C29" s="17" t="s">
+        <v>64</v>
+      </c>
+      <c r="D29" s="17">
+        <v>5</v>
+      </c>
+      <c r="E29" s="24" t="str">
+        <f t="shared" si="3"/>
+        <v>Vincent Eric Leumann/1. Platz,</v>
+      </c>
+      <c r="F29" s="25">
+        <f>_xlfn.XLOOKUP(D29,'Bewertung Projekte'!$C$23:$J$23,'Bewertung Projekte'!$C$36:$J$36)</f>
+        <v>3</v>
+      </c>
+      <c r="G29" s="24" t="str">
+        <f t="shared" si="4"/>
+        <v>3. Platz</v>
+      </c>
+      <c r="H29" s="24" t="str">
+        <f t="shared" si="2"/>
+        <v>{herausragendes }</v>
+      </c>
+      <c r="I29" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="J29" s="20"/>
+      <c r="K29" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="H4" s="16">
-        <f>146.25/(A16+2)</f>
-        <v>9.140625</v>
-      </c>
-      <c r="I4" s="14" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A5" s="6">
-        <v>3</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" s="8" t="s">
+    </row>
+    <row r="30" spans="1:11" ht="17" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A30" s="21">
         <v>12</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="B30" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="C30" s="17" t="s">
+        <v>66</v>
+      </c>
+      <c r="D30" s="17">
+        <v>6</v>
+      </c>
+      <c r="E30" s="24" t="str">
+        <f t="shared" si="3"/>
+        <v>Nour el Zahra Mostafa/1. Platz,</v>
+      </c>
+      <c r="F30" s="25">
+        <f>_xlfn.XLOOKUP(D30,'Bewertung Projekte'!$C$23:$J$23,'Bewertung Projekte'!$C$36:$J$36)</f>
+        <v>8</v>
+      </c>
+      <c r="G30" s="24" t="str">
+        <f t="shared" si="4"/>
+        <v>Honorable Mention</v>
+      </c>
+      <c r="H30" s="24" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="I30" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="J30" s="20"/>
+    </row>
+    <row r="31" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A31" s="21">
+        <v>13</v>
+      </c>
+      <c r="B31" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="C31" s="17" t="s">
+        <v>68</v>
+      </c>
+      <c r="D31" s="17">
+        <v>1</v>
+      </c>
+      <c r="E31" s="24" t="str">
+        <f t="shared" si="3"/>
+        <v>Lenny Schnetzer/1. Platz,</v>
+      </c>
+      <c r="F31" s="25">
+        <f>_xlfn.XLOOKUP(D31,'Bewertung Projekte'!$C$23:$J$23,'Bewertung Projekte'!$C$36:$J$36)</f>
+        <v>1</v>
+      </c>
+      <c r="G31" s="24" t="str">
+        <f t="shared" si="4"/>
+        <v>1. Platz</v>
+      </c>
+      <c r="H31" s="24" t="str">
+        <f t="shared" si="2"/>
+        <v>{herausragendes }</v>
+      </c>
+      <c r="I31" s="18" t="s">
+        <v>69</v>
+      </c>
+      <c r="J31" s="20"/>
+    </row>
+    <row r="32" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A32" s="21">
+        <v>14</v>
+      </c>
+      <c r="B32" s="16" t="s">
+        <v>70</v>
+      </c>
+      <c r="C32" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="D32" s="17">
+        <v>4</v>
+      </c>
+      <c r="E32" s="24" t="str">
+        <f t="shared" si="3"/>
+        <v>Tom Schnyder/1. Platz,</v>
+      </c>
+      <c r="F32" s="25">
+        <f>_xlfn.XLOOKUP(D32,'Bewertung Projekte'!$C$23:$J$23,'Bewertung Projekte'!$C$36:$J$36)</f>
+        <v>2</v>
+      </c>
+      <c r="G32" s="24" t="str">
+        <f t="shared" si="4"/>
+        <v>2. Platz</v>
+      </c>
+      <c r="H32" s="24" t="str">
+        <f t="shared" si="2"/>
+        <v>{herausragendes }</v>
+      </c>
+      <c r="I32" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="J32" s="20"/>
+    </row>
+    <row r="33" spans="1:10" ht="17" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A33" s="21">
+        <v>15</v>
+      </c>
+      <c r="B33" s="16" t="s">
+        <v>72</v>
+      </c>
+      <c r="C33" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="D33" s="17">
+        <v>2</v>
+      </c>
+      <c r="E33" s="24" t="str">
+        <f t="shared" si="3"/>
+        <v>Filippo Straumann/1. Platz,</v>
+      </c>
+      <c r="F33" s="25">
+        <f>_xlfn.XLOOKUP(D33,'Bewertung Projekte'!$C$23:$J$23,'Bewertung Projekte'!$C$36:$J$36)</f>
+        <v>4</v>
+      </c>
+      <c r="G33" s="24" t="str">
+        <f t="shared" si="4"/>
+        <v>Honorable Mention</v>
+      </c>
+      <c r="H33" s="24" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="I33" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="J33" s="20"/>
+    </row>
+    <row r="34" spans="1:10" ht="18.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A34" s="21">
+        <v>16</v>
+      </c>
+      <c r="B34" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="C34" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="D34" s="17">
+        <v>4</v>
+      </c>
+      <c r="E34" s="24" t="str">
+        <f t="shared" si="3"/>
+        <v>Yannick Widler/1. Platz,</v>
+      </c>
+      <c r="F34" s="25">
+        <f>_xlfn.XLOOKUP(D34,'Bewertung Projekte'!$C$23:$J$23,'Bewertung Projekte'!$C$36:$J$36)</f>
+        <v>2</v>
+      </c>
+      <c r="G34" s="24" t="str">
+        <f t="shared" si="4"/>
+        <v>2. Platz</v>
+      </c>
+      <c r="H34" s="24" t="str">
+        <f t="shared" si="2"/>
+        <v>{herausragendes }</v>
+      </c>
+      <c r="I34" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="J34" s="20"/>
+    </row>
+    <row r="35" spans="1:10" ht="18.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A35" s="21">
+        <v>17</v>
+      </c>
+      <c r="B35" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="C35" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="D35" s="17">
         <v>7</v>
       </c>
-      <c r="E5" s="11" t="s">
-        <v>76</v>
-      </c>
-      <c r="H5" s="16">
-        <v>15</v>
-      </c>
-      <c r="I5" s="14" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A6" s="6">
-        <v>4</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="D6" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="E6" s="11" t="s">
-        <v>76</v>
-      </c>
-      <c r="H6" s="16">
-        <f>SUM(H3:H5)</f>
-        <v>29.140625</v>
-      </c>
-      <c r="I6" s="14" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A7" s="6">
-        <v>5</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="D7" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="E7" s="11" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A8" s="6">
+      <c r="E35" s="24" t="str">
+        <f t="shared" si="3"/>
+        <v>Daniil Domashenko/1. Platz,</v>
+      </c>
+      <c r="F35" s="25">
+        <f>_xlfn.XLOOKUP(D35,'Bewertung Projekte'!$C$23:$J$23,'Bewertung Projekte'!$C$36:$J$36)</f>
         <v>6</v>
       </c>
-      <c r="B8" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="D8" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="E8" s="1"/>
-    </row>
-    <row r="9" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A9" s="6">
-        <v>7</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="D9" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="E9" s="11" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A10" s="6">
-        <v>8</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="C10" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="D10" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="E10" s="11" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A11" s="6">
-        <v>9</v>
-      </c>
-      <c r="B11" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="D11" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="E11" s="11" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A12" s="10">
-        <v>10</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="C12" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="D12" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="E12" s="11" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A13" s="10">
-        <v>11</v>
-      </c>
-      <c r="B13" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="C13" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="D13" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="E13" s="11" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A14" s="10">
-        <v>12</v>
-      </c>
-      <c r="B14" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="C14" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="D14" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="E14" s="11" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A15" s="10">
-        <v>13</v>
-      </c>
-      <c r="B15" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="C15" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="D15" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="E15" s="11" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A16" s="10">
-        <v>14</v>
-      </c>
-      <c r="B16" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="C16" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="D16" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="E16" s="11" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" ht="48" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A17" s="13" t="s">
-        <v>37</v>
-      </c>
-      <c r="B17" s="13"/>
-      <c r="C17" s="13"/>
-      <c r="D17" s="13"/>
-      <c r="E17" s="13"/>
-      <c r="H17" s="17" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A18" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="E18" s="1"/>
-      <c r="H18" s="15">
-        <v>5</v>
-      </c>
-      <c r="I18" s="14" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A19" s="6">
-        <v>1</v>
-      </c>
-      <c r="B19" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="C19" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="D19" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="E19" s="1"/>
-      <c r="H19" s="16">
-        <f>146.25/(A35+2)</f>
-        <v>7.6973684210526319</v>
-      </c>
-      <c r="I19" s="14" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A20" s="6">
-        <v>2</v>
-      </c>
-      <c r="B20" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="C20" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="D20" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="E20" s="1"/>
-      <c r="H20" s="16">
-        <v>15</v>
-      </c>
-      <c r="I20" s="14" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A21" s="6">
-        <v>3</v>
-      </c>
-      <c r="B21" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="C21" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="D21" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="E21" s="1"/>
-      <c r="H21" s="16">
-        <f>SUM(H18:H20)</f>
-        <v>27.69736842105263</v>
-      </c>
-      <c r="I21" s="14" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A22" s="6">
-        <v>4</v>
-      </c>
-      <c r="B22" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="C22" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="D22" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="E22" s="1"/>
-    </row>
-    <row r="23" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A23" s="6">
-        <v>5</v>
-      </c>
-      <c r="B23" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="C23" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="D23" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="E23" s="1"/>
-    </row>
-    <row r="24" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A24" s="6">
-        <v>6</v>
-      </c>
-      <c r="B24" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="C24" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="D24" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="E24" s="1"/>
-    </row>
-    <row r="25" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A25" s="6">
-        <v>7</v>
-      </c>
-      <c r="B25" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="C25" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="D25" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="E25" s="1"/>
-    </row>
-    <row r="26" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A26" s="6">
-        <v>8</v>
-      </c>
-      <c r="B26" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="C26" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="D26" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="E26" s="1"/>
-    </row>
-    <row r="27" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A27" s="6">
-        <v>9</v>
-      </c>
-      <c r="B27" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="C27" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="D27" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="E27" s="1"/>
-    </row>
-    <row r="28" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A28" s="10">
-        <v>10</v>
-      </c>
-      <c r="B28" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="C28" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="D28" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="E28" s="1"/>
-    </row>
-    <row r="29" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A29" s="10">
-        <v>11</v>
-      </c>
-      <c r="B29" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="C29" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="D29" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="E29" s="1"/>
-      <c r="F29" s="14" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A30" s="10">
-        <v>12</v>
-      </c>
-      <c r="B30" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="C30" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="D30" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="E30" s="1"/>
-    </row>
-    <row r="31" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A31" s="10">
-        <v>13</v>
-      </c>
-      <c r="B31" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="C31" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="D31" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="E31" s="1"/>
-    </row>
-    <row r="32" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A32" s="10">
-        <v>14</v>
-      </c>
-      <c r="B32" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="C32" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="D32" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="E32" s="1"/>
-    </row>
-    <row r="33" spans="1:5" ht="17" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A33" s="10">
-        <v>15</v>
-      </c>
-      <c r="B33" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="C33" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="D33" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="E33" s="1"/>
-    </row>
-    <row r="34" spans="1:5" ht="18.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A34" s="10">
-        <v>16</v>
-      </c>
-      <c r="B34" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="C34" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="D34" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="E34" s="1"/>
-    </row>
-    <row r="35" spans="1:5" ht="18.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A35" s="10">
-        <v>17</v>
-      </c>
-      <c r="B35" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="C35" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="D35" s="9" t="s">
+      <c r="G35" s="24" t="str">
+        <f t="shared" si="4"/>
+        <v>Honorable Mention</v>
+      </c>
+      <c r="H35" s="24" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="I35" s="18" t="s">
         <v>80</v>
       </c>
-      <c r="E35" s="1"/>
+      <c r="J35" s="20"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A17:E17"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A17:J17"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{487C5AB6-1562-574B-8E26-E259D3429CAC}">
+  <dimension ref="A1:R36"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
+  <cols>
+    <col min="1" max="1" width="6" customWidth="1"/>
+    <col min="2" max="2" width="26.3984375" customWidth="1"/>
+    <col min="3" max="3" width="15.3984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.19921875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.59765625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.3984375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:18" x14ac:dyDescent="0.15">
+      <c r="A1" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.15">
+      <c r="C2" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.15">
+      <c r="A3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B3" t="s">
+        <v>88</v>
+      </c>
+      <c r="C3" s="1">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>2</v>
+      </c>
+      <c r="E3" s="1">
+        <v>3</v>
+      </c>
+      <c r="F3">
+        <v>4</v>
+      </c>
+      <c r="G3">
+        <v>5</v>
+      </c>
+      <c r="H3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.15">
+      <c r="A4" s="1">
+        <v>1</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="C4" s="1">
+        <v>1</v>
+      </c>
+      <c r="D4" s="1">
+        <v>1</v>
+      </c>
+      <c r="E4" s="1">
+        <v>0</v>
+      </c>
+      <c r="F4" s="1">
+        <v>1</v>
+      </c>
+      <c r="G4" s="1">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>1</v>
+      </c>
+      <c r="I4" s="1"/>
+      <c r="J4" s="1"/>
+      <c r="K4" s="1"/>
+      <c r="L4" s="1"/>
+      <c r="M4" s="1"/>
+      <c r="N4" s="1"/>
+      <c r="O4" s="1"/>
+      <c r="P4" s="1"/>
+      <c r="Q4" s="1"/>
+      <c r="R4" s="1"/>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.15">
+      <c r="A5" s="1">
+        <v>1</v>
+      </c>
+      <c r="B5" t="s">
+        <v>91</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>0.5</v>
+      </c>
+      <c r="E5" s="1">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>0.5</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.15">
+      <c r="A6" s="1">
+        <v>1</v>
+      </c>
+      <c r="B6" t="s">
+        <v>92</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6" s="1">
+        <v>0</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.15">
+      <c r="A7" s="1">
+        <v>1</v>
+      </c>
+      <c r="B7" t="s">
+        <v>93</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7" s="1">
+        <v>1</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7">
+        <v>1</v>
+      </c>
+      <c r="H7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.15">
+      <c r="A8" s="1">
+        <v>1</v>
+      </c>
+      <c r="B8" t="s">
+        <v>94</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8" s="1">
+        <v>1</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
+      </c>
+      <c r="G8">
+        <v>1</v>
+      </c>
+      <c r="H8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.15">
+      <c r="A9" s="1">
+        <v>1</v>
+      </c>
+      <c r="B9" t="s">
+        <v>95</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9" s="1">
+        <v>1</v>
+      </c>
+      <c r="F9">
+        <v>1</v>
+      </c>
+      <c r="G9">
+        <v>1</v>
+      </c>
+      <c r="H9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.15">
+      <c r="A10" s="1">
+        <v>1</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10" s="1">
+        <v>0</v>
+      </c>
+      <c r="F10">
+        <v>0</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.15">
+      <c r="A11" s="1">
+        <v>2</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C11">
+        <v>0.5</v>
+      </c>
+      <c r="D11">
+        <v>0.5</v>
+      </c>
+      <c r="E11" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="F11" s="27">
+        <v>1.5</v>
+      </c>
+      <c r="G11">
+        <v>2</v>
+      </c>
+      <c r="H11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.15">
+      <c r="A12" s="1">
+        <v>2</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="C12">
+        <v>1</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12" s="1">
+        <v>0</v>
+      </c>
+      <c r="F12">
+        <v>1</v>
+      </c>
+      <c r="G12">
+        <v>2</v>
+      </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.15">
+      <c r="A13" s="1">
+        <v>2</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="C13">
+        <v>0</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13" s="1">
+        <v>0</v>
+      </c>
+      <c r="F13">
+        <v>1</v>
+      </c>
+      <c r="G13">
+        <v>0</v>
+      </c>
+      <c r="H13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.15">
+      <c r="A14" s="1">
+        <v>1</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C14" s="1">
+        <v>1</v>
+      </c>
+      <c r="D14">
+        <v>1</v>
+      </c>
+      <c r="E14" s="1">
+        <v>1</v>
+      </c>
+      <c r="F14" s="1">
+        <v>1</v>
+      </c>
+      <c r="G14">
+        <v>1</v>
+      </c>
+      <c r="H14" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.15">
+      <c r="A15">
+        <f>SUM(A4:A14)</f>
+        <v>14</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="C15" s="5">
+        <f>SUM(C4:C14)</f>
+        <v>9.5</v>
+      </c>
+      <c r="D15" s="5">
+        <f>SUM(D4:D14)</f>
+        <v>6</v>
+      </c>
+      <c r="E15" s="5">
+        <f>SUM(E4:E14)</f>
+        <v>4.5</v>
+      </c>
+      <c r="F15" s="5">
+        <f>SUM(F4:F14)</f>
+        <v>10</v>
+      </c>
+      <c r="G15" s="5">
+        <f>SUM(G4:G14)</f>
+        <v>11</v>
+      </c>
+      <c r="H15" s="5">
+        <f>SUM(H4:H14)</f>
+        <v>7.5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.15">
+      <c r="B16" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="C16">
+        <f t="shared" ref="C16:F16" si="0">RANK(C15,$C$15:$H$15)</f>
+        <v>3</v>
+      </c>
+      <c r="D16">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="E16" s="1">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="F16">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="G16">
+        <f>RANK(G15,$C$15:$H$15)</f>
+        <v>1</v>
+      </c>
+      <c r="H16">
+        <f t="shared" ref="H16" si="1">RANK(H15,$C$15:$H$15)</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.15">
+      <c r="A21" s="1" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.15">
+      <c r="C22" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.15">
+      <c r="A23" t="s">
+        <v>89</v>
+      </c>
+      <c r="B23" t="s">
+        <v>88</v>
+      </c>
+      <c r="C23" s="1">
+        <v>1</v>
+      </c>
+      <c r="D23">
+        <v>2</v>
+      </c>
+      <c r="E23" s="1">
+        <v>3</v>
+      </c>
+      <c r="F23">
+        <v>4</v>
+      </c>
+      <c r="G23">
+        <v>5</v>
+      </c>
+      <c r="H23">
+        <v>6</v>
+      </c>
+      <c r="I23">
+        <v>7</v>
+      </c>
+      <c r="J23">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.15">
+      <c r="A24" s="1">
+        <v>1</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="C24" s="1"/>
+      <c r="D24" s="1"/>
+      <c r="E24" s="1"/>
+      <c r="F24" s="1"/>
+      <c r="G24" s="1"/>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.15">
+      <c r="A25" s="1">
+        <v>1</v>
+      </c>
+      <c r="B25" t="s">
+        <v>91</v>
+      </c>
+      <c r="E25" s="1"/>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.15">
+      <c r="A26" s="1">
+        <v>1</v>
+      </c>
+      <c r="B26" t="s">
+        <v>92</v>
+      </c>
+      <c r="E26" s="1"/>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.15">
+      <c r="A27" s="1">
+        <v>1</v>
+      </c>
+      <c r="B27" t="s">
+        <v>93</v>
+      </c>
+      <c r="E27" s="1"/>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.15">
+      <c r="A28" s="1">
+        <v>1</v>
+      </c>
+      <c r="B28" t="s">
+        <v>94</v>
+      </c>
+      <c r="E28" s="1"/>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.15">
+      <c r="A29" s="1">
+        <v>1</v>
+      </c>
+      <c r="B29" t="s">
+        <v>95</v>
+      </c>
+      <c r="E29" s="1"/>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.15">
+      <c r="A30" s="1">
+        <v>1</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="E30" s="1"/>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.15">
+      <c r="A31" s="1">
+        <v>2</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C31">
+        <v>5443</v>
+      </c>
+      <c r="D31">
+        <v>9</v>
+      </c>
+      <c r="E31" s="1">
+        <v>8</v>
+      </c>
+      <c r="F31" s="27">
+        <v>77</v>
+      </c>
+      <c r="G31">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.15">
+      <c r="A32" s="1">
+        <v>2</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="E32" s="1"/>
+      <c r="G32">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.15">
+      <c r="A33" s="1">
+        <v>2</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="E33" s="1"/>
+      <c r="G33">
+        <v>6</v>
+      </c>
+      <c r="I33">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.15">
+      <c r="A34" s="1">
+        <v>1</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C34" s="1"/>
+      <c r="E34" s="1"/>
+      <c r="F34" s="1"/>
+      <c r="H34" s="1"/>
+      <c r="J34">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.15">
+      <c r="A35">
+        <f>SUM(A24:A34)</f>
+        <v>14</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="C35" s="5">
+        <f>SUM(C24:C34)</f>
+        <v>5443</v>
+      </c>
+      <c r="D35" s="5">
+        <f>SUM(D24:D34)</f>
+        <v>9</v>
+      </c>
+      <c r="E35" s="5">
+        <f>SUM(E24:E34)</f>
+        <v>8</v>
+      </c>
+      <c r="F35" s="5">
+        <f>SUM(F24:F34)</f>
+        <v>77</v>
+      </c>
+      <c r="G35" s="5">
+        <f>SUM(G24:G34)</f>
+        <v>20</v>
+      </c>
+      <c r="H35" s="5">
+        <f>SUM(H24:H34)</f>
+        <v>0</v>
+      </c>
+      <c r="I35" s="5">
+        <f>SUM(I24:I34)</f>
+        <v>5</v>
+      </c>
+      <c r="J35" s="5">
+        <f>SUM(J24:J34)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.15">
+      <c r="B36" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="C36">
+        <f t="shared" ref="C36:I36" si="2">RANK(C35,$C$35:$J$35)</f>
+        <v>1</v>
+      </c>
+      <c r="D36">
+        <f t="shared" si="2"/>
+        <v>4</v>
+      </c>
+      <c r="E36">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="F36">
+        <f t="shared" si="2"/>
+        <v>2</v>
+      </c>
+      <c r="G36">
+        <f t="shared" si="2"/>
+        <v>3</v>
+      </c>
+      <c r="H36">
+        <f t="shared" si="2"/>
+        <v>8</v>
+      </c>
+      <c r="I36">
+        <f t="shared" si="2"/>
+        <v>6</v>
+      </c>
+      <c r="J36">
+        <f>RANK(J35,$C$35:$J$35)</f>
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBD3BA99-117A-BA4C-87EB-B3D531E59314}">
+  <dimension ref="A1:B20"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A1" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A2" s="2">
+        <v>5</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A3" s="3">
+        <f>146.25/(TN!A16+2)</f>
+        <v>9.140625</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A4" s="3">
+        <v>15</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A5" s="3">
+        <f>SUM(A2:A4)</f>
+        <v>29.140625</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A16" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A17" s="2">
+        <v>5</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A18" s="3">
+        <f>146.25/(TN!A35+2)</f>
+        <v>7.6973684210526319</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A19" s="3">
+        <v>15</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A20" s="3">
+        <f>SUM(A17:A19)</f>
+        <v>27.69736842105263</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>85</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>